<commit_message>
Fix rugs image issue
</commit_message>
<xml_diff>
--- a/ICR Work Complete.xlsx
+++ b/ICR Work Complete.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="19">
   <si>
     <t>✅ Next.js deployed</t>
   </si>
@@ -70,6 +70,9 @@
   </si>
   <si>
     <t>Complete</t>
+  </si>
+  <si>
+    <t>Half way</t>
   </si>
 </sst>
 </file>
@@ -507,6 +510,9 @@
       <c r="A12" s="1" t="s">
         <v>10</v>
       </c>
+      <c r="B12" s="1" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">

</xml_diff>